<commit_message>
refactor: modernisation exceptions, safe_ui_action, couverture tests 60.73%
</commit_message>
<xml_diff>
--- a/example/example_RE/reverse_sample.xlsx
+++ b/example/example_RE/reverse_sample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lemarchand\Mon Drive\couches minces 2026\CERTUS\2003\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lemarchand\Mon Drive\couches minces 2026\CERTUS\1705\example\example_RE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D555231E-94B1-47A5-82C5-71B8988E270B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCFDC45D-BCAF-4389-B678-1703CBA2D36F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="1920" windowWidth="32352" windowHeight="14688" activeTab="1" xr2:uid="{FD9746D7-B3C0-446F-B840-FEBDFC0AB19F}"/>
+    <workbookView xWindow="4152" yWindow="1212" windowWidth="36924" windowHeight="14688" activeTab="1" xr2:uid="{FD9746D7-B3C0-446F-B840-FEBDFC0AB19F}"/>
   </bookViews>
   <sheets>
     <sheet name="measurement" sheetId="1" r:id="rId1"/>
@@ -41,9 +41,6 @@
     <t>lambda</t>
   </si>
   <si>
-    <t xml:space="preserve">silicon </t>
-  </si>
-  <si>
     <t>Wavelength, nm</t>
   </si>
   <si>
@@ -66,6 +63,9 @@
   </si>
   <si>
     <t>R-45p-noBK</t>
+  </si>
+  <si>
+    <t>silicon</t>
   </si>
 </sst>
 </file>
@@ -464,13 +464,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -7102,7 +7102,7 @@
         <v>1500</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -7201,7 +7201,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" style="1"/>
-    <col min="2" max="2" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="27.33203125" bestFit="1" customWidth="1"/>
@@ -7209,19 +7209,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>